<commit_message>
Refactor engine into modular processing pipeline
</commit_message>
<xml_diff>
--- a/data/healthy.xlsx
+++ b/data/healthy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pratham OS\Development\Finance-AI\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B9C1C4B-D9DE-409A-9C34-3283B565FA04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84F774D1-00AE-4D9F-AE6B-DE57849672A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="855" firstSheet="3" activeTab="3" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="855" firstSheet="3" activeTab="11" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
@@ -2434,7 +2434,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
         <v>86</v>
       </c>

</xml_diff>

<commit_message>
Backend Architecture Complete | Finance AI v0.9.9
</commit_message>
<xml_diff>
--- a/data/healthy.xlsx
+++ b/data/healthy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pratham OS\Development\Finance-AI\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84F774D1-00AE-4D9F-AE6B-DE57849672A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E3AFC84-1F6F-4F41-9AC4-DF0CA417AF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="855" firstSheet="3" activeTab="11" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
+    <workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="8880" tabRatio="855" firstSheet="2" activeTab="2" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
@@ -1231,12 +1231,6 @@
   </cellStyles>
   <dxfs count="32">
     <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
       <font>
         <color rgb="FF9C0006"/>
       </font>
@@ -1258,6 +1252,18 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
@@ -1329,6 +1335,12 @@
       </font>
     </dxf>
     <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
     </dxf>
     <dxf>
@@ -1339,6 +1351,9 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1383,21 +1398,6 @@
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1412,14 +1412,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="25" tableBorderDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="30" tableBorderDxfId="29">
   <autoFilter ref="A1:H1048576" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date" dataDxfId="23"/>
+    <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date" dataDxfId="28"/>
     <tableColumn id="4" xr3:uid="{E805A8A8-660D-4099-912A-BE1B697553ED}" name="Type"/>
     <tableColumn id="5" xr3:uid="{ABF1E4D7-7922-479D-94F4-994DCBA1062D}" name="Category"/>
     <tableColumn id="6" xr3:uid="{E21EA904-BC60-4EB5-B4BD-249E5A12FC76}" name="Description "/>
-    <tableColumn id="7" xr3:uid="{EFA172CE-B81A-4A83-BB09-0C52BED62422}" name="Amount" dataDxfId="22"/>
+    <tableColumn id="7" xr3:uid="{EFA172CE-B81A-4A83-BB09-0C52BED62422}" name="Amount" dataDxfId="27"/>
     <tableColumn id="8" xr3:uid="{E811D3EB-DAD5-46D9-B70D-01072B332F5C}" name="Need/Want"/>
     <tableColumn id="9" xr3:uid="{1E8766C9-2C6F-4CE3-9C7E-C6C8545D3945}" name="Payment Mode"/>
     <tableColumn id="10" xr3:uid="{BA26CD78-BAFB-4644-808D-0A18546F6CAF}" name="Recurring"/>
@@ -1432,9 +1432,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{204CD917-42D7-44E9-889E-B87F7E170616}" name="Table5" displayName="Table5" ref="A1:C100" totalsRowShown="0">
   <autoFilter ref="A1:C100" xr:uid="{204CD917-42D7-44E9-889E-B87F7E170616}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CCD99EA9-9CA0-4F69-8282-1EE2E5FE7967}" name="Month" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{CCD99EA9-9CA0-4F69-8282-1EE2E5FE7967}" name="Month" dataDxfId="26"/>
     <tableColumn id="2" xr3:uid="{5C307EC1-8BAE-4B8C-AF42-D468202B7A5E}" name="Year"/>
-    <tableColumn id="3" xr3:uid="{2B3569FD-9348-4E00-BFEA-53DF4F58E82C}" name="Monthly_Budget" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{2B3569FD-9348-4E00-BFEA-53DF4F58E82C}" name="Monthly_Budget" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1444,40 +1444,40 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}" name="FinancialCommitments" displayName="FinancialCommitments" ref="A1:K45" totalsRowShown="0">
   <autoFilter ref="A1:K45" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Start Date " dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Start Date " dataDxfId="24"/>
     <tableColumn id="2" xr3:uid="{D6130D6E-B2EE-4D09-94CD-7E8053CD1C7B}" name="From"/>
     <tableColumn id="3" xr3:uid="{8ECD20EB-BEF0-47D5-8DA5-28D491EC7B0A}" name="Type"/>
-    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Total Amount" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Total Amount" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="21"/>
     <tableColumn id="7" xr3:uid="{FFDA91C5-2668-4023-9FEE-465A59D85270}" name="Due Date"/>
     <tableColumn id="8" xr3:uid="{748EB09B-78B0-49AB-AC7E-88A7F4C42C89}" name="Status"/>
     <tableColumn id="10" xr3:uid="{39DD9F5E-EB31-47B4-A27F-BDA3AA61DA00}" name="commitment"/>
-    <tableColumn id="11" xr3:uid="{740721D4-21BC-47E8-A178-052DE413178D}" name="Monthly Payment" dataDxfId="0"/>
-    <tableColumn id="12" xr3:uid="{2EEE087F-37EF-44B3-8405-6F6CCBE4BDEB}" name="End Date" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{740721D4-21BC-47E8-A178-052DE413178D}" name="Monthly Payment" dataDxfId="20"/>
+    <tableColumn id="12" xr3:uid="{2EEE087F-37EF-44B3-8405-6F6CCBE4BDEB}" name="End Date" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <autoFilter ref="A1:G4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{ED3F2086-7429-4708-9751-1D0D42E41B00}" name="Table6" displayName="Table6" ref="A1:H4" totalsRowShown="0" headerRowDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{ED3F2086-7429-4708-9751-1D0D42E41B00}" name="Table6" displayName="Table6" ref="A1:H4" totalsRowShown="0" headerRowDxfId="9">
   <autoFilter ref="A1:H4" xr:uid="{ED3F2086-7429-4708-9751-1D0D42E41B00}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{02A819B9-5B65-4731-BA10-C393EA3AE4AE}" name="Goal"/>
@@ -1497,7 +1497,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{7E348894-AB6B-47ED-8D66-B030107418E7}" name="Table7" displayName="Table7" ref="A1:J200" totalsRowShown="0">
   <autoFilter ref="A1:J200" xr:uid="{7E348894-AB6B-47ED-8D66-B030107418E7}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{76E56D66-576D-4754-ADFE-436DD70011B2}" name="Date" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{76E56D66-576D-4754-ADFE-436DD70011B2}" name="Date" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{AAAC6B22-EF0E-43D9-B017-EB668B0236DD}" name="Investment"/>
     <tableColumn id="3" xr3:uid="{CF097674-7777-4A04-A504-F67ED104098F}" name="Type"/>
     <tableColumn id="4" xr3:uid="{1C676C24-A4B4-439F-AF8F-F0507E28FD4D}" name="Platform"/>
@@ -1518,12 +1518,12 @@
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{1BF6EFB3-081D-479F-97D0-5D410AC21987}" name="Liability"/>
     <tableColumn id="9" xr3:uid="{0B74D237-DA90-49D5-A8A6-285DE9F93208}" name="Category"/>
-    <tableColumn id="2" xr3:uid="{63AF3204-721F-4930-9003-E0E2451D091B}" name="Original Loan" dataDxfId="31"/>
-    <tableColumn id="3" xr3:uid="{271A520E-175A-4E77-8ACA-00A70E60B367}" name="Outstanding Balance" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{4AC64920-C6E6-4621-AC5A-DBB95F045FB6}" name="Monthly EMI" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{EA313BB7-3226-4263-8B2A-D21A5A3EC593}" name="Intrest %" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{E47C1A29-AD81-4EC2-9222-0D1F1C94F36D}" name="Start Date" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{5A74DAD1-ED79-464B-A2CB-CFDC6117FC4F}" name="End Date" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{63AF3204-721F-4930-9003-E0E2451D091B}" name="Original Loan" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{271A520E-175A-4E77-8ACA-00A70E60B367}" name="Outstanding Balance" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{4AC64920-C6E6-4621-AC5A-DBB95F045FB6}" name="Monthly EMI" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{EA313BB7-3226-4263-8B2A-D21A5A3EC593}" name="Intrest %" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{E47C1A29-AD81-4EC2-9222-0D1F1C94F36D}" name="Start Date" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{5A74DAD1-ED79-464B-A2CB-CFDC6117FC4F}" name="End Date" dataDxfId="2"/>
     <tableColumn id="8" xr3:uid="{6232A2AD-0FD7-4B56-A36F-A1E8D77D37A2}" name="Status"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1538,7 +1538,7 @@
     <tableColumn id="2" xr3:uid="{AC7352C6-0DC7-4AFC-BDAD-303C389924A5}" name="Category"/>
     <tableColumn id="3" xr3:uid="{9884F549-FF9E-426C-A41E-5854163D6493}" name="Purchase Value"/>
     <tableColumn id="4" xr3:uid="{486852BE-C51C-4E3A-9B66-11D7D9CCEE9B}" name="Current Value"/>
-    <tableColumn id="5" xr3:uid="{2F141C2F-956F-436C-B98A-F15A4A0A762D}" name="Purchase Date" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{2F141C2F-956F-436C-B98A-F15A4A0A762D}" name="Purchase Date" dataDxfId="31"/>
     <tableColumn id="6" xr3:uid="{ED74E306-AFE5-436F-911F-2ED2CC19D23C}" name="Status"/>
     <tableColumn id="7" xr3:uid="{93FAD5D9-55A0-4F40-A483-B99C6367CC93}" name="Notes"/>
   </tableColumns>
@@ -2075,10 +2075,10 @@
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <conditionalFormatting sqref="B17:B20">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2388,7 +2388,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>83</v>
       </c>
@@ -2411,7 +2411,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="18" t="s">
         <v>304</v>
       </c>
@@ -2457,7 +2457,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="s">
         <v>307</v>
       </c>
@@ -2480,7 +2480,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="18" t="s">
         <v>309</v>
       </c>
@@ -4747,7 +4747,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2">
         <v>2026</v>
@@ -5288,7 +5288,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="20">
         <v>46218</v>
       </c>
@@ -5311,7 +5311,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="20">
         <v>46223</v>
       </c>

</xml_diff>